<commit_message>
Recolor spreadsheet CV in the Altarism palette
Ember bands, oxblood intro and headings, plum links, palette tab colors. README points to the Google Sheet copy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spreadsheet-resume/viv-tran-cv.xlsx
+++ b/spreadsheet-resume/viv-tran-cv.xlsx
@@ -35,35 +35,41 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00F6F3EC"/>
       <sz val="20"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="006E413A"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00F6F3EC"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00180F06"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00180F06"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00755367"/>
       <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
+      <color rgb="00180F06"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,11 +78,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="006E413A"/>
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid"/>
+      <patternFill patternType="solid">
+        <fgColor rgb="00180F06"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6F3EC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -89,21 +102,21 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00180F06"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00180F06"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00180F06"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00180F06"/>
       </bottom>
     </border>
     <border>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00180F06"/>
       </top>
     </border>
   </borders>
@@ -123,13 +136,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -501,6 +514,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="006E413A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -525,6 +539,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00755367"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -663,6 +678,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B77C45"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1360,6 +1376,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00566B47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1450,6 +1467,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00AAA7A1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1726,6 +1744,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00180F06"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1844,6 +1863,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="006E413A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2046,6 +2066,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00755367"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2181,6 +2202,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B77C45"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>